<commit_message>
fab(rev6): guide-compliant crystal spec (10pF CL) + L1 orientation note
JLCPCB flagged crystal + polarised inductor vs the RP2350 design guide:
- Y1 = 12MHz 3225 CL=10pF (ABM8-272-T3 class) w/ the 15pF caps - rev5's
  20pF-load crystal would run off-tune with 15pF caps. BOM-only change.
- L1: RP2350 SMPS inductor is polarity-sensitive (guide Figure); pick a
  marked part, order remark 'dot toward U1'. Board uses no ADC -> low
  practical risk, but documented for the assembler.
</commit_message>
<xml_diff>
--- a/hardware/fab-rev6/imspi8080-rev6-bom.xlsx
+++ b/hardware/fab-rev6/imspi8080-rev6-bom.xlsx
@@ -424,7 +424,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="5" customWidth="1" min="4" max="4"/>
-    <col width="31" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="70" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
   </cols>
@@ -543,7 +543,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>12MHz crystal</t>
+          <t>12MHz crystal (10pF load)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -563,12 +563,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12MHz 20pF</t>
+          <t>12MHz 3225 4P 10pF (ABM8-272-T3 class)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Core clock. Basic. Load caps C_Y1a/b.</t>
+          <t>RP2350 guide crystal: 12MHz, CL=10pF, with 15pF load caps C23/C24. Do NOT use a 20pF-load crystal here (rev5's part) - it would run off-tune.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">

</xml_diff>

<commit_message>
fab(rev6): L1 = SMNR4020-2.2UH C135262 (4040, 3.4A/3.4A, 46mOhm)
Selected in JLCPCB picker after stock check; 4x4mm lands inside the
5.2mm SRU5016-pattern pads. Crystal line still pending the user's pick.
</commit_message>
<xml_diff>
--- a/hardware/fab-rev6/imspi8080-rev6-bom.xlsx
+++ b/hardware/fab-rev6/imspi8080-rev6-bom.xlsx
@@ -422,7 +422,7 @@
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="5" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="70" customWidth="1" min="6" max="6"/>
@@ -3702,7 +3702,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>L_Bourns-SRU5016 5.2x5.2mm</t>
+          <t>SMD 4x4mm (4040)</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -3712,15 +3712,19 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>2.2uH 5.2x5.2 shielded &gt;=1.5A</t>
+          <t>SMNR4020-2.2UH</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>RP2350 VREG DC-DC inductor: VREG_LX to VREG_FB (VCORE). REQUIRED for RP2350 core rail.</t>
-        </is>
-      </c>
-      <c r="G97" t="inlineStr"/>
+          <t>RP2350 VREG DC-DC inductor: VREG_LX to VREG_FB (VCORE). 3.4A/3.4A, 46mOhm. Orient marking toward U1.</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>C135262</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fab(rev6): Y1 = ABM8-272-T3 C20625731 - the guide crystal
Exact Raspberry Pi RP2350 hardware-design-guide part (12MHz, 3225-4P,
CL=10pF, 50ohm, +-30ppm). BOM fully resolved: U1 RP2350A C42411118,
L1 SMNR4020-2R2UH C135262, Y1 ABM8-272-T3 C20625731.
</commit_message>
<xml_diff>
--- a/hardware/fab-rev6/imspi8080-rev6-bom.xlsx
+++ b/hardware/fab-rev6/imspi8080-rev6-bom.xlsx
@@ -424,7 +424,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="5" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="70" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
   </cols>
@@ -543,7 +543,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>12MHz crystal (10pF load)</t>
+          <t>12MHz crystal</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -553,7 +553,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SMD-3225-4P</t>
+          <t>SMD3225-4P</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -563,17 +563,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>12MHz 3225 4P 10pF (ABM8-272-T3 class)</t>
+          <t>ABM8-272-T3</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>RP2350 guide crystal: 12MHz, CL=10pF, with 15pF load caps C23/C24. Do NOT use a 20pF-load crystal here (rev5's part) - it would run off-tune.</t>
+          <t>EXACT RP2350 hardware-design-guide crystal: 12MHz, 3225-4P, CL=10pF, 50ohm ESR, +-30ppm. With 15pF C23/C24.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>C9002</t>
+          <t>C20625731</t>
         </is>
       </c>
     </row>

</xml_diff>